<commit_message>
committed @ 2025-10-24-095855-0500 by tcn85@rtsjpl774kw20.managed.mst.edu
</commit_message>
<xml_diff>
--- a/data/3420-2025-fall-quizzes/3420-2025-fall-quizzzes.xlsx
+++ b/data/3420-2025-fall-quizzes/3420-2025-fall-quizzzes.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tcn85/workspace/dsm/data/3420-2025-fall-quizzes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C5DCEE3-ABC7-CB4A-9773-ED669B550586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E66DB001-5B47-1E43-A1B7-315AC5A51749}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25920" yWindow="-1340" windowWidth="25920" windowHeight="20980" activeTab="2" xr2:uid="{02943BD8-8D23-1D42-A928-8937731C9A90}"/>
+    <workbookView xWindow="-38400" yWindow="-1340" windowWidth="16640" windowHeight="20980" activeTab="4" xr2:uid="{02943BD8-8D23-1D42-A928-8937731C9A90}"/>
   </bookViews>
   <sheets>
-    <sheet name="py-np-pd-2" sheetId="4" r:id="rId1"/>
-    <sheet name="py-np-pd" sheetId="3" r:id="rId2"/>
-    <sheet name="py-review" sheetId="2" r:id="rId3"/>
-    <sheet name="py-review(OLD)" sheetId="1" r:id="rId4"/>
+    <sheet name="midterm" sheetId="5" r:id="rId1"/>
+    <sheet name="py-np-pd-2" sheetId="4" r:id="rId2"/>
+    <sheet name="py-np-pd" sheetId="3" r:id="rId3"/>
+    <sheet name="py-review" sheetId="2" r:id="rId4"/>
+    <sheet name="py-review(OLD)" sheetId="1" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="62">
   <si>
     <t>name</t>
   </si>
@@ -222,6 +223,9 @@
   </si>
   <si>
     <t>q1.1.for loop with function</t>
+  </si>
+  <si>
+    <t>quiz_ID</t>
   </si>
 </sst>
 </file>
@@ -603,6 +607,350 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CB7E6D7-60B8-2742-BB3B-0032338A8090}">
+  <dimension ref="A2:O24"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="7.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="3.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3">
+        <v>50</v>
+      </c>
+      <c r="O3" s="2"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4">
+        <v>50</v>
+      </c>
+      <c r="O4" s="2"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5">
+        <v>46</v>
+      </c>
+      <c r="O5" s="2"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6">
+        <v>50</v>
+      </c>
+      <c r="O6" s="2"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7">
+        <v>50</v>
+      </c>
+      <c r="O7" s="2"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8">
+        <v>48</v>
+      </c>
+      <c r="O8" s="2"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>45</v>
+      </c>
+      <c r="O9" s="2"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10">
+        <v>48</v>
+      </c>
+      <c r="O10" s="2"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11">
+        <v>50</v>
+      </c>
+      <c r="O11" s="2"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12">
+        <v>47</v>
+      </c>
+      <c r="O12" s="2"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13">
+        <v>50</v>
+      </c>
+      <c r="O13" s="2"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>20</v>
+      </c>
+      <c r="B14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" t="s">
+        <v>55</v>
+      </c>
+      <c r="O14" s="2"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>17</v>
+      </c>
+      <c r="B15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15">
+        <v>48</v>
+      </c>
+      <c r="O15" s="2"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>11</v>
+      </c>
+      <c r="B16" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16">
+        <v>46</v>
+      </c>
+      <c r="O16" s="2"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>5</v>
+      </c>
+      <c r="B17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17">
+        <v>38</v>
+      </c>
+      <c r="O17" s="2"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>1</v>
+      </c>
+      <c r="B18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18">
+        <v>48</v>
+      </c>
+      <c r="O18" s="2"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>9</v>
+      </c>
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" t="s">
+        <v>42</v>
+      </c>
+      <c r="D19">
+        <v>45</v>
+      </c>
+      <c r="O19" s="2"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>10</v>
+      </c>
+      <c r="B20" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20">
+        <v>48</v>
+      </c>
+      <c r="O20" s="2"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>8</v>
+      </c>
+      <c r="B21" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21">
+        <v>48</v>
+      </c>
+      <c r="O21" s="2"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>4</v>
+      </c>
+      <c r="B22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" t="s">
+        <v>40</v>
+      </c>
+      <c r="D22">
+        <v>50</v>
+      </c>
+      <c r="O22" s="2"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B008A34-68DC-614D-9212-709EBD2097C8}">
   <dimension ref="A2:J24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1390,7 +1738,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{625988FA-08F2-5D4B-BCDA-BABB71AA94B0}">
   <dimension ref="A2:K24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2242,7 +2590,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C470603-E249-6C49-AFDF-564C1138E589}">
   <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3380,7 +3728,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{253F1E1C-F588-7C4E-B050-53E91BB391E3}">
   <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>